<commit_message>
Page qui se fige après inactivité : préchargement des morceaux d'interface stlite ; changement de chantier sans anciens fichiers ; colonne TL ; Textile : Qté sur étagère dans les tableaux, Prévision en dernier
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QT8GhHjeho8wXovFt7nryP
</commit_message>
<xml_diff>
--- a/tests/fixtures/etat_stock.xlsx
+++ b/tests/fixtures/etat_stock.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U17"/>
+  <dimension ref="A1:V17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -565,6 +565,11 @@
           <t>DATE DERNIERE CONSO</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>TRACKING LEVEL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -640,6 +645,11 @@
       <c r="U2" s="1" t="n">
         <v>46266</v>
       </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>TL1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -715,6 +725,11 @@
       <c r="U3" s="1" t="n">
         <v>46266</v>
       </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>TL0</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -790,6 +805,11 @@
       <c r="U4" s="1" t="n">
         <v>46296</v>
       </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>TL1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -865,6 +885,11 @@
       <c r="U5" s="1" t="n">
         <v>46266</v>
       </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>TL0</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -940,6 +965,11 @@
       <c r="U6" s="1" t="n">
         <v>46266</v>
       </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>TL1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1015,6 +1045,11 @@
       <c r="U7" s="1" t="n">
         <v>46266</v>
       </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>TL0</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1090,6 +1125,11 @@
       <c r="U8" s="1" t="n">
         <v>46266</v>
       </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>TL0</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1160,6 +1200,11 @@
       <c r="U9" s="1" t="n">
         <v>46266</v>
       </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>TL0</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1235,6 +1280,11 @@
       <c r="U10" s="1" t="n">
         <v>46266</v>
       </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>TL0</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1310,6 +1360,11 @@
       <c r="U11" s="1" t="n">
         <v>46266</v>
       </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>TL0</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1384,6 +1439,11 @@
       </c>
       <c r="U12" s="1" t="n">
         <v>46266</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>TL1</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1458,6 +1518,11 @@
       <c r="U13" s="1" t="n">
         <v>46266</v>
       </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>TL0</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1533,6 +1598,11 @@
       <c r="U14" s="1" t="n">
         <v>46266</v>
       </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>TL0</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1608,6 +1678,11 @@
       <c r="U15" s="1" t="n">
         <v>46266</v>
       </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>TL1</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1683,6 +1758,11 @@
       <c r="U16" s="1" t="n">
         <v>43586</v>
       </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>TL1</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1757,6 +1837,11 @@
       </c>
       <c r="U17" s="1" t="n">
         <v>36892</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>TL0</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Onglet PE mousses : objectif de l'année (Besoin Prod) × stock × commandes par CCN, avions faisables avec répartition des CCN communs, avions restants recalculés avec le fichier PE mousses ; Avancement PE et Forecast déplacés depuis le Textile
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QT8GhHjeho8wXovFt7nryP
</commit_message>
<xml_diff>
--- a/tests/fixtures/etat_stock.xlsx
+++ b/tests/fixtures/etat_stock.xlsx
@@ -1880,7 +1880,7 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>60</v>
+        <v>7101</v>
       </c>
       <c r="J18" t="n">
         <v>1</v>
@@ -1960,7 +1960,7 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>60</v>
+        <v>7102</v>
       </c>
       <c r="J19" t="n">
         <v>1</v>
@@ -2040,7 +2040,7 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>60</v>
+        <v>7103</v>
       </c>
       <c r="J20" t="n">
         <v>1</v>
@@ -2120,7 +2120,7 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>60</v>
+        <v>7104</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
@@ -2200,7 +2200,7 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>60</v>
+        <v>7201</v>
       </c>
       <c r="J22" t="n">
         <v>1</v>
@@ -2280,7 +2280,7 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>60</v>
+        <v>7202</v>
       </c>
       <c r="J23" t="n">
         <v>1</v>
@@ -2360,7 +2360,7 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>60</v>
+        <v>7203</v>
       </c>
       <c r="J24" t="n">
         <v>1</v>

</xml_diff>